<commit_message>
DHCP DNS atirasa SW+kliens ip-k hozzaadasa
</commit_message>
<xml_diff>
--- a/NagyTet-kft.Topologia ip cimek es protokollok.xlsx
+++ b/NagyTet-kft.Topologia ip cimek es protokollok.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\peterd\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07A026BF-4301-41A3-B12B-BE7134E8CAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD6872EA-8FD3-4133-ADAD-C590C46E7279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{406C4712-5E1D-4CD4-9337-AA77B4CD174F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="133">
   <si>
     <t>Routerek</t>
   </si>
@@ -161,9 +161,6 @@
     <t>192.168.15.1</t>
   </si>
   <si>
-    <t>ipv6</t>
-  </si>
-  <si>
     <t>192.168.21.1</t>
   </si>
   <si>
@@ -356,15 +353,9 @@
     <t>192.168.24.11</t>
   </si>
   <si>
-    <t>192.168.24.12</t>
-  </si>
-  <si>
     <t>Fa0/9</t>
   </si>
   <si>
-    <t>Fa0/10</t>
-  </si>
-  <si>
     <t>192.168.34.99</t>
   </si>
   <si>
@@ -389,12 +380,6 @@
     <t>HSRP Virtual 192.168.25.1</t>
   </si>
   <si>
-    <t>DNS</t>
-  </si>
-  <si>
-    <t>LINUX</t>
-  </si>
-  <si>
     <t>Tuzfal</t>
   </si>
   <si>
@@ -402,13 +387,61 @@
   </si>
   <si>
     <t>Gig1/2</t>
+  </si>
+  <si>
+    <t>192.168.16.1</t>
+  </si>
+  <si>
+    <t>192.168.17.1</t>
+  </si>
+  <si>
+    <t>GAME_Belepo_SW</t>
+  </si>
+  <si>
+    <t>Fa0/1-3</t>
+  </si>
+  <si>
+    <t>2001:db8:15::1/64</t>
+  </si>
+  <si>
+    <t>2001:db8:16::1/64</t>
+  </si>
+  <si>
+    <t>2001:db8:17::1/64</t>
+  </si>
+  <si>
+    <t>DUAL STACK IPV4 IPV6</t>
+  </si>
+  <si>
+    <t>10.10.10.5</t>
+  </si>
+  <si>
+    <t>10.10.10.6</t>
+  </si>
+  <si>
+    <t>10.10.10.41</t>
+  </si>
+  <si>
+    <t>10.10.10.42</t>
+  </si>
+  <si>
+    <t>10.10.10.37</t>
+  </si>
+  <si>
+    <t>10.10.10.38</t>
+  </si>
+  <si>
+    <t>Linux_DHCP</t>
+  </si>
+  <si>
+    <t>Windows_DNS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -429,6 +462,13 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -458,7 +498,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -481,11 +521,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -499,11 +548,20 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -840,76 +898,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D6C8071-E3A0-431C-AEBD-FB6269738AF3}">
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.85546875" customWidth="1"/>
-    <col min="2" max="2" width="22.28515625" customWidth="1"/>
+    <col min="2" max="2" width="41.7109375" customWidth="1"/>
     <col min="3" max="3" width="24.42578125" customWidth="1"/>
     <col min="4" max="4" width="31" style="1" customWidth="1"/>
-    <col min="5" max="5" width="24.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" customWidth="1"/>
     <col min="6" max="6" width="28.85546875" customWidth="1"/>
     <col min="7" max="7" width="23.7109375" customWidth="1"/>
     <col min="8" max="8" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.140625" customWidth="1"/>
+    <col min="10" max="10" width="24.42578125" customWidth="1"/>
     <col min="11" max="11" width="25.7109375" customWidth="1"/>
     <col min="12" max="12" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>87</v>
+        <v>18</v>
       </c>
       <c r="G1" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="I1" s="1"/>
       <c r="J1" s="3" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="K1" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
+      <c r="B2" s="1" t="s">
+        <v>125</v>
+      </c>
       <c r="C2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="F2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="I2" s="1"/>
-      <c r="J2" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="L2" t="s">
-        <v>72</v>
-      </c>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -922,23 +982,23 @@
         <v>11</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>66</v>
+        <v>19</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="K3" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="I3" s="1"/>
-      <c r="J3" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="L3" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -955,23 +1015,23 @@
         <v>32</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="I4" s="1"/>
-      <c r="J4" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="L4" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -988,23 +1048,23 @@
         <v>33</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="G5" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L5" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="I5" s="1"/>
-      <c r="J5" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L5" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1021,22 +1081,22 @@
         <v>34</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>74</v>
+        <v>25</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="H6" s="1"/>
+        <v>21</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="I6" s="1"/>
-      <c r="J6" s="5" t="s">
-        <v>21</v>
+      <c r="J6" s="1" t="s">
+        <v>73</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="L6" t="s">
-        <v>72</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -1051,24 +1111,24 @@
       <c r="D7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="L7" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="I7" s="1"/>
-      <c r="J7" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="L7" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -1076,127 +1136,135 @@
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="L8" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="1"/>
-      <c r="J8" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="L8" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>41</v>
+      <c r="B9" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="H9" s="5" t="s">
         <v>12</v>
       </c>
+      <c r="F9" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>24</v>
+      </c>
       <c r="I9" s="1"/>
-      <c r="J9" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="K9" s="6"/>
-      <c r="L9" t="s">
-        <v>120</v>
+      <c r="J9" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="4"/>
+        <v>2</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>117</v>
+      </c>
       <c r="C10" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>120</v>
       </c>
       <c r="I10" s="1"/>
-      <c r="J10" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="K10" s="6"/>
-      <c r="L10" t="s">
-        <v>121</v>
-      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>50</v>
+        <v>2</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>118</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>120</v>
       </c>
       <c r="I11" s="1"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>51</v>
+        <v>3</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>130</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>86</v>
+        <v>12</v>
       </c>
       <c r="I12" s="1"/>
+      <c r="J12" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>20</v>
+        <v>10</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K13" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -1204,526 +1272,558 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>24</v>
+        <v>11</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="K14" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="4"/>
+      <c r="B15" s="1" t="s">
+        <v>51</v>
+      </c>
       <c r="C15" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>22</v>
+        <v>91</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>23</v>
+        <v>99</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="K15" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>22</v>
+        <v>91</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>55</v>
+        <v>4</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>127</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>116</v>
-      </c>
       <c r="F17" s="1" t="s">
-        <v>25</v>
+        <v>92</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>21</v>
+        <v>101</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>116</v>
-      </c>
       <c r="F20" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+        <v>100</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="L21" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="L22" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H22" s="1" t="s">
+      <c r="F23" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H23" s="1" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J23" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="L23" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="K24" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="L24" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C25" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="L25" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="J26" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="K26" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="L26" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="D27" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G25" s="1" t="s">
+      <c r="F27" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="L27" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="K28" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="L28" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="G29" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="H29" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H30" s="1" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B27" s="1" t="s">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G28" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="H28" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C29" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G30" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="H30" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="F31" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
+        <v>32</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C33" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="D35" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G33" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C34" s="1" t="s">
+      <c r="B36" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F34" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C35" s="1" t="s">
+      <c r="B37" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F35" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F36" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F37" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F38" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H38" s="1" t="s">
-        <v>100</v>
-      </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F39" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="H39" s="1" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F40" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H40" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F42" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="F45" s="1"/>
-      <c r="G45" s="1"/>
-      <c r="H45" s="1"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="J12:L12"/>
+  </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>

</xml_diff>